<commit_message>
Sample upload: accept numeric region codes 1-13 (NUTS-2 order)
Survey Solutions codes the region as a number 1-13 in NUTS-2 code order.

- sample_io.py: add REGION_NUM map and number-based stratum matching alongside
  Greek name and EL.. code. Template Reference tab now lists No. + Region + Code
  in NUTS-2 order; instructions note the 1-13 option.
- README updated.

https://claude.ai/code/session_01UKT8V6ygx7iYZ4q6CUYW6c
</commit_message>
<xml_diff>
--- a/oecd_tracker/templates/Sample_Daily_Responses_Template.xlsx
+++ b/oecd_tracker/templates/Sample_Daily_Responses_Template.xlsx
@@ -486,7 +486,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • Region (NUTS-2)   — Greek name OR EL.. code (see Reference tab)</t>
+          <t xml:space="preserve">    • Region (NUTS-2)   — number 1-13, EL.. code, or Greek name (see Reference tab)</t>
         </is>
       </c>
     </row>
@@ -574,185 +574,230 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Valid Region values (name or code)</t>
+          <t>Valid Region values — use the No., the Code, or the name</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
           <t>Region (NUTS-2)</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Αττική</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>EL30</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Βόρειο Αιγαίο</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EL41</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Νότιο Αιγαίο</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>EL42</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Κρήτη</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>EL43</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ανατολική Μακεδονία και Θράκη</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>EL51</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Κεντρική Μακεδονία</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>EL52</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Δυτική Μακεδονία</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>EL53</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ήπειρος</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EL54</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Θεσσαλία</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>EL61</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ιόνια Νησιά</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>EL62</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Δυτική Ελλάδα</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>EL63</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Κρήτη</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>EL43</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Ανατολική Μακεδονία και Θράκη</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>EL51</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Στερεά Ελλάδα</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>EL64</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>Πελοπόννησος</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>EL65</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Ήπειρος</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>EL54</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Νότιο Αιγαίο</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>EL42</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Δυτική Μακεδονία</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>EL53</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Βόρειο Αιγαίο</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>EL41</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Ιόνια Νησιά</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>EL62</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sample upload: real QD2 region codes + QD3 urbanity collapse
Use the actual Survey Solutions codebook instead of assumed orderings.

- Region (QD2): codes 1-13 in the questionnaire's order (08 = Στερεά Ελλάδα /
  "Κεντρικής Ελλάδας"); -97/-99 (don't know / no answer) excluded.
- Urbanity (QD3): 5 settlement sizes collapsed to the 2 strata — 3,4,5 (>=15k)
  = Αστικά; 1,2 = Αγροτικά/Ημιαστικά. Numeric codes parsed; Greek/English labels
  still accepted.
- Template Reference tab documents both QD2 and QD3 mappings; instructions and
  README updated; excluded-row caption clarified.

https://claude.ai/code/session_01UKT8V6ygx7iYZ4q6CUYW6c
</commit_message>
<xml_diff>
--- a/oecd_tracker/templates/Sample_Daily_Responses_Template.xlsx
+++ b/oecd_tracker/templates/Sample_Daily_Responses_Template.xlsx
@@ -486,14 +486,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • Region (NUTS-2)   — number 1-13, EL.. code, or Greek name (see Reference tab)</t>
+          <t xml:space="preserve">    • Region   — QD2 code 1-13 (or EL.. code / Greek name; see Reference tab). -97/-99 are excluded.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • Urban/Rural   — Αστικά or Αγροτικά/Ημιαστικά (Urban/Rural also ok)</t>
+          <t xml:space="preserve">    • Urban/Rural   — QD3 code 1-5: 3,4,5 = Αστικά; 1,2 = Αγροτικά/Ημιαστικά.</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
   <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
@@ -585,24 +585,24 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Valid Region values — use the No., the Code, or the name</t>
+          <t>Region — QD2 code, or EL.. code, or name</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>No.</t>
+          <t>QD2</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Region (NUTS-2)</t>
+          <t>Region</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>EL code</t>
         </is>
       </c>
     </row>
@@ -627,12 +627,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Βόρειο Αιγαίο</t>
+          <t>Κεντρική Μακεδονία</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>EL41</t>
+          <t>EL52</t>
         </is>
       </c>
     </row>
@@ -642,12 +642,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Νότιο Αιγαίο</t>
+          <t>Θεσσαλία</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>EL42</t>
+          <t>EL61</t>
         </is>
       </c>
     </row>
@@ -657,12 +657,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Κρήτη</t>
+          <t>Δυτική Ελλάδα</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>EL43</t>
+          <t>EL63</t>
         </is>
       </c>
     </row>
@@ -672,12 +672,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ανατολική Μακεδονία και Θράκη</t>
+          <t>Κρήτη</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>EL51</t>
+          <t>EL43</t>
         </is>
       </c>
     </row>
@@ -687,12 +687,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Κεντρική Μακεδονία</t>
+          <t>Ανατολική Μακεδονία και Θράκη</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>EL52</t>
+          <t>EL51</t>
         </is>
       </c>
     </row>
@@ -702,12 +702,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Δυτική Μακεδονία</t>
+          <t>Πελοπόννησος</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>EL53</t>
+          <t>EL65</t>
         </is>
       </c>
     </row>
@@ -717,12 +717,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ήπειρος</t>
+          <t>Στερεά Ελλάδα</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>EL54</t>
+          <t>EL64</t>
         </is>
       </c>
     </row>
@@ -732,12 +732,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Θεσσαλία</t>
+          <t>Ήπειρος</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>EL61</t>
+          <t>EL54</t>
         </is>
       </c>
     </row>
@@ -747,12 +747,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Ιόνια Νησιά</t>
+          <t>Νότιο Αιγαίο</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>EL62</t>
+          <t>EL42</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Δυτική Ελλάδα</t>
+          <t>Δυτική Μακεδονία</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>EL63</t>
+          <t>EL53</t>
         </is>
       </c>
     </row>
@@ -777,12 +777,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Στερεά Ελλάδα</t>
+          <t>Ιόνια Νησιά</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>EL64</t>
+          <t>EL62</t>
         </is>
       </c>
     </row>
@@ -792,31 +792,41 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Πελοπόννησος</t>
+          <t>Βόρειο Αιγαίο</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>EL65</t>
+          <t>EL41</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Valid Urban/Rural values</t>
+          <t>Urban/Rural — QD3 code → stratum</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>3, 4, 5</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>Αστικά</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>Αγροτικά/Ημιαστικά</t>
         </is>

</xml_diff>